<commit_message>
docs: sincronizar planificación oficial de BeautyOS
</commit_message>
<xml_diff>
--- a/docs/beautyos/BeautyOS_Cronograma_Maestro.xlsx
+++ b/docs/beautyos/BeautyOS_Cronograma_Maestro.xlsx
@@ -2869,59 +2869,239 @@
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" ht="15">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Decisiones aprobadas</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="15">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Mobile-first</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Operaciones diarias priorizan celular; toda UI futura se valida en móvil/tablet/desktop y móvil puede usar flujos simplificados.</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="15">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Identidad Core</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>User es la identidad; Student, Professional e Instructor son perfiles/relaciones. Student→Graduate→Professional no duplica identidad.</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="26" spans="1:9" ht="15">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Producto y Core</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>BeautyOS es comercializable independientemente, puede reutilizar Core y no depende de módulos exclusivos MVS. Core preparado para productos combinables o independientes.</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="15">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Privacidad Academy</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Academy conoce solo su relación educativa y señal profesional autorizada; nunca datos privados del negocio del egresado por esa relación.</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="15">
       <c r="A28" s="1"/>
@@ -2935,15 +3115,51 @@
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" ht="15">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Academy por fases</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>Core → Importación/aprobación → Student Hub → Lab → Certificación/Graduate Network → Knowledge AI/Brand Knowledge/Templates.</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="15">
       <c r="A30" s="1"/>
@@ -2957,15 +3173,51 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" ht="15">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Hipótesis comercial</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>Academy Founder/Partner, subsidio inicial, límites de almacenamiento/IA y créditos por activación voluntaria requieren validación; no son precios definitivos.</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="32" spans="1:9" ht="15">
       <c r="A32" s="1"/>
@@ -3527,13 +3779,19 @@
         <v>113</v>
       </c>
       <c r="K9" s="3"/>
-      <c r="L9" s="3" t="s">
-        <v>54</v>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
       </c>
       <c r="M9" s="6">
-        <v>0</v>
-      </c>
-      <c r="N9" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Confirmado por commit d74aad6; modelos Professional/Specialty, migración, fábricas y prueba BeautyProfessionalSpecialtyTest. B06 no iniciado.</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="1:14" ht="27">
       <c r="A10" s="3" t="s">
@@ -3695,129 +3953,201 @@
       </c>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:14" ht="15">
-      <c r="A14" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>146</v>
+    <row r="14" spans="1:14" ht="27">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>B79</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Arquitectura transversal</t>
+        </is>
       </c>
       <c r="C14" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4">
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="E14" s="4">
-        <v>46278</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3" t="s">
-        <v>54</v>
+        <v>46271</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Formalizar estándar mobile-first multiformato</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Criterio transversal aprobado: operaciones diarias priorizan celular; cada UI se valida en móvil/tablet/desktop y puede ofrecer flujos móviles simplificados</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>B01-B09</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M14" s="6">
         <v>0</v>
       </c>
-      <c r="N14" s="3"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Decisión aprobada; no inicia implementación</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:14" ht="27">
-      <c r="A15" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>146</v>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Arquitectura transversal</t>
+        </is>
       </c>
       <c r="C15" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" s="4">
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="E15" s="4">
-        <v>46278</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3" t="s">
-        <v>54</v>
+        <v>46271</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Formalizar identidad Core y perfiles BeautyOS</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Modelo aprobado: User es identidad Core; Student, Professional e Instructor son perfiles/relaciones sin identidad duplicada; transición Student→Graduate→Professional preserva identidad</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Mixto</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>B03-B05</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M15" s="6">
         <v>0</v>
       </c>
-      <c r="N15" s="3"/>
-    </row>
-    <row r="16" spans="1:14" ht="15">
-      <c r="A16" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>146</v>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Decisión aprobada; B05 permanece completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="27">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>B81</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Arquitectura transversal</t>
+        </is>
       </c>
       <c r="C16" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4">
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="E16" s="4">
-        <v>46278</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3" t="s">
-        <v>54</v>
+        <v>46271</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Definir independencia comercial y límites del Core compartido</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>BeautyOS vendible independientemente, reutiliza Core sin depender de módulos exclusivos MVS; Core preparado para RRHH, Contabilidad, TallerOS y productos futuros</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Mixto</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>B01-B04</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M16" s="6">
         <v>0</v>
       </c>
-      <c r="N16" s="3"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Decisión aprobada; exige multiempresa/multisucursal estricto</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:14" ht="15">
       <c r="A17" s="3" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>146</v>
@@ -3832,19 +4162,19 @@
         <v>46278</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="s">
@@ -3857,31 +4187,31 @@
     </row>
     <row r="18" spans="1:14" ht="27">
       <c r="A18" s="3" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>146</v>
       </c>
       <c r="C18" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" s="4">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="E18" s="4">
-        <v>46285</v>
+        <v>46278</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>113</v>
@@ -3897,34 +4227,34 @@
     </row>
     <row r="19" spans="1:14" ht="15">
       <c r="A19" s="3" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>146</v>
       </c>
       <c r="C19" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D19" s="4">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="E19" s="4">
-        <v>46285</v>
+        <v>46278</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="3" t="s">
@@ -3935,33 +4265,33 @@
       </c>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="27">
+    <row r="20" spans="1:14" ht="15">
       <c r="A20" s="3" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>146</v>
       </c>
       <c r="C20" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20" s="4">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="E20" s="4">
-        <v>46285</v>
+        <v>46278</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>51</v>
@@ -3975,9 +4305,9 @@
       </c>
       <c r="N20" s="3"/>
     </row>
-    <row r="21" spans="1:14" ht="15">
+    <row r="21" spans="1:14" ht="27">
       <c r="A21" s="3" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>146</v>
@@ -3992,16 +4322,16 @@
         <v>46285</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>173</v>
+        <v>133</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>113</v>
@@ -4015,33 +4345,33 @@
       </c>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" ht="27">
+    <row r="22" spans="1:14" ht="15">
       <c r="A22" s="3" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="C22" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="4">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="E22" s="4">
-        <v>46292</v>
+        <v>46285</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>113</v>
@@ -4055,36 +4385,36 @@
       </c>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" ht="15">
+    <row r="23" spans="1:14" ht="27">
       <c r="A23" s="3" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="C23" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="4">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="E23" s="4">
-        <v>46292</v>
+        <v>46285</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="3" t="s">
@@ -4097,31 +4427,31 @@
     </row>
     <row r="24" spans="1:14" ht="15">
       <c r="A24" s="3" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="C24" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="4">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="E24" s="4">
-        <v>46292</v>
+        <v>46285</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>113</v>
@@ -4135,9 +4465,9 @@
       </c>
       <c r="N24" s="3"/>
     </row>
-    <row r="25" spans="1:14" ht="15">
+    <row r="25" spans="1:14" ht="27">
       <c r="A25" s="3" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>175</v>
@@ -4152,19 +4482,19 @@
         <v>46292</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3" t="s">
@@ -4177,31 +4507,31 @@
     </row>
     <row r="26" spans="1:14" ht="15">
       <c r="A26" s="3" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>175</v>
       </c>
       <c r="C26" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" s="4">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="E26" s="4">
-        <v>46299</v>
+        <v>46292</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>191</v>
+        <v>174</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>113</v>
@@ -4217,34 +4547,34 @@
     </row>
     <row r="27" spans="1:14" ht="15">
       <c r="A27" s="3" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>175</v>
       </c>
       <c r="C27" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27" s="4">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="E27" s="4">
-        <v>46299</v>
+        <v>46292</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3" t="s">
@@ -4255,33 +4585,33 @@
       </c>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="27">
+    <row r="28" spans="1:14" ht="15">
       <c r="A28" s="3" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>175</v>
       </c>
       <c r="C28" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" s="4">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="E28" s="4">
-        <v>46299</v>
+        <v>46292</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>111</v>
+        <v>165</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>51</v>
@@ -4295,9 +4625,9 @@
       </c>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="27">
+    <row r="29" spans="1:14" ht="15">
       <c r="A29" s="3" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>175</v>
@@ -4312,19 +4642,19 @@
         <v>46299</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="s">
@@ -4335,9 +4665,9 @@
       </c>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="27">
+    <row r="30" spans="1:14" ht="15">
       <c r="A30" s="3" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>175</v>
@@ -4352,19 +4682,19 @@
         <v>46299</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="s">
@@ -4375,33 +4705,33 @@
       </c>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="15">
+    <row r="31" spans="1:14" ht="27">
       <c r="A31" s="3" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>206</v>
+        <v>175</v>
       </c>
       <c r="C31" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D31" s="4">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="E31" s="4">
-        <v>46306</v>
+        <v>46299</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>51</v>
@@ -4417,25 +4747,25 @@
     </row>
     <row r="32" spans="1:14" ht="27">
       <c r="A32" s="3" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>206</v>
+        <v>175</v>
       </c>
       <c r="C32" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D32" s="4">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="E32" s="4">
-        <v>46306</v>
+        <v>46299</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>117</v>
@@ -4457,34 +4787,34 @@
     </row>
     <row r="33" spans="1:14" ht="27">
       <c r="A33" s="3" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>206</v>
+        <v>175</v>
       </c>
       <c r="C33" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D33" s="4">
-        <v>46307</v>
+        <v>46293</v>
       </c>
       <c r="E33" s="4">
-        <v>46313</v>
+        <v>46299</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="3" t="s">
@@ -4495,27 +4825,27 @@
       </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" ht="27">
+    <row r="34" spans="1:14" ht="15">
       <c r="A34" s="3" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>206</v>
       </c>
       <c r="C34" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D34" s="4">
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="E34" s="4">
-        <v>46313</v>
+        <v>46306</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>117</v>
@@ -4524,7 +4854,7 @@
         <v>192</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3" t="s">
@@ -4535,27 +4865,27 @@
       </c>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="15">
+    <row r="35" spans="1:14" ht="27">
       <c r="A35" s="3" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>206</v>
       </c>
       <c r="C35" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D35" s="4">
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="E35" s="4">
-        <v>46313</v>
+        <v>46306</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>117</v>
@@ -4564,7 +4894,7 @@
         <v>192</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3" t="s">
@@ -4577,34 +4907,34 @@
     </row>
     <row r="36" spans="1:14" ht="27">
       <c r="A36" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>206</v>
       </c>
       <c r="C36" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D36" s="4">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="E36" s="4">
-        <v>46320</v>
+        <v>46313</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>224</v>
+        <v>192</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3" t="s">
@@ -4617,34 +4947,34 @@
     </row>
     <row r="37" spans="1:14" ht="27">
       <c r="A37" s="3" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>206</v>
       </c>
       <c r="C37" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D37" s="4">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="E37" s="4">
-        <v>46320</v>
+        <v>46313</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3" t="s">
@@ -4655,36 +4985,36 @@
       </c>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="27">
+    <row r="38" spans="1:14" ht="15">
       <c r="A38" s="3" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>206</v>
       </c>
       <c r="C38" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D38" s="4">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="E38" s="4">
-        <v>46320</v>
+        <v>46313</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>232</v>
+        <v>192</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="3" t="s">
@@ -4695,33 +5025,33 @@
       </c>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="15">
+    <row r="39" spans="1:14" ht="27">
       <c r="A39" s="3" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="C39" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D39" s="4">
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="E39" s="4">
-        <v>46327</v>
+        <v>46320</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>235</v>
+        <v>222</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>236</v>
+        <v>223</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>167</v>
+        <v>224</v>
       </c>
       <c r="J39" s="3" t="s">
         <v>113</v>
@@ -4737,31 +5067,31 @@
     </row>
     <row r="40" spans="1:14" ht="27">
       <c r="A40" s="3" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="C40" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D40" s="4">
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="E40" s="4">
-        <v>46327</v>
+        <v>46320</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="J40" s="3" t="s">
         <v>51</v>
@@ -4775,33 +5105,33 @@
       </c>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="15">
+    <row r="41" spans="1:14" ht="27">
       <c r="A41" s="3" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="C41" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D41" s="4">
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="E41" s="4">
-        <v>46327</v>
+        <v>46320</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>165</v>
+        <v>117</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="J41" s="3" t="s">
         <v>51</v>
@@ -4815,9 +5145,9 @@
       </c>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="27">
+    <row r="42" spans="1:14" ht="15">
       <c r="A42" s="3" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>234</v>
@@ -4832,19 +5162,19 @@
         <v>46327</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>233</v>
+        <v>167</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3" t="s">
@@ -4857,34 +5187,34 @@
     </row>
     <row r="43" spans="1:14" ht="27">
       <c r="A43" s="3" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>234</v>
       </c>
       <c r="C43" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D43" s="4">
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="E43" s="4">
-        <v>46334</v>
+        <v>46327</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="3" t="s">
@@ -4895,33 +5225,33 @@
       </c>
       <c r="N43" s="3"/>
     </row>
-    <row r="44" spans="1:14" ht="27">
+    <row r="44" spans="1:14" ht="15">
       <c r="A44" s="3" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>234</v>
       </c>
       <c r="C44" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D44" s="4">
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="E44" s="4">
-        <v>46334</v>
+        <v>46327</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="J44" s="3" t="s">
         <v>51</v>
@@ -4935,36 +5265,36 @@
       </c>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="15">
+    <row r="45" spans="1:14" ht="27">
       <c r="A45" s="3" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>234</v>
       </c>
       <c r="C45" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D45" s="4">
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="E45" s="4">
-        <v>46334</v>
+        <v>46327</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>233</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="3" t="s">
@@ -4975,9 +5305,9 @@
       </c>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="15">
+    <row r="46" spans="1:14" ht="27">
       <c r="A46" s="3" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>234</v>
@@ -4992,16 +5322,16 @@
         <v>46334</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="J46" s="3" t="s">
         <v>113</v>
@@ -5015,33 +5345,33 @@
       </c>
       <c r="N46" s="3"/>
     </row>
-    <row r="47" spans="1:14" ht="15">
+    <row r="47" spans="1:14" ht="27">
       <c r="A47" s="3" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>262</v>
+        <v>234</v>
       </c>
       <c r="C47" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D47" s="4">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="E47" s="4">
-        <v>46341</v>
+        <v>46334</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="H47" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="J47" s="3" t="s">
         <v>51</v>
@@ -5057,31 +5387,31 @@
     </row>
     <row r="48" spans="1:14" ht="15">
       <c r="A48" s="3" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>262</v>
+        <v>234</v>
       </c>
       <c r="C48" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D48" s="4">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="E48" s="4">
-        <v>46341</v>
+        <v>46334</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>261</v>
+        <v>233</v>
       </c>
       <c r="J48" s="3" t="s">
         <v>113</v>
@@ -5095,36 +5425,36 @@
       </c>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" ht="27">
+    <row r="49" spans="1:14" ht="15">
       <c r="A49" s="3" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>262</v>
+        <v>234</v>
       </c>
       <c r="C49" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D49" s="4">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="E49" s="4">
-        <v>46341</v>
+        <v>46334</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>159</v>
+        <v>260</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K49" s="3"/>
       <c r="L49" s="3" t="s">
@@ -5137,34 +5467,34 @@
     </row>
     <row r="50" spans="1:14" ht="15">
       <c r="A50" s="3" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>262</v>
       </c>
       <c r="C50" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" s="4">
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="E50" s="4">
-        <v>46348</v>
+        <v>46341</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="3" t="s">
@@ -5177,31 +5507,31 @@
     </row>
     <row r="51" spans="1:14" ht="15">
       <c r="A51" s="3" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>262</v>
       </c>
       <c r="C51" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D51" s="4">
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="E51" s="4">
-        <v>46348</v>
+        <v>46341</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="J51" s="3" t="s">
         <v>113</v>
@@ -5217,31 +5547,31 @@
     </row>
     <row r="52" spans="1:14" ht="27">
       <c r="A52" s="3" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>262</v>
       </c>
       <c r="C52" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D52" s="4">
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="E52" s="4">
-        <v>46348</v>
+        <v>46341</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>283</v>
+        <v>159</v>
       </c>
       <c r="J52" s="3" t="s">
         <v>51</v>
@@ -5257,7 +5587,7 @@
     </row>
     <row r="53" spans="1:14" ht="15">
       <c r="A53" s="3" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>262</v>
@@ -5272,19 +5602,19 @@
         <v>46348</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="3" t="s">
@@ -5297,34 +5627,34 @@
     </row>
     <row r="54" spans="1:14" ht="15">
       <c r="A54" s="3" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>288</v>
+        <v>262</v>
       </c>
       <c r="C54" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D54" s="4">
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="E54" s="4">
-        <v>46355</v>
+        <v>46348</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>127</v>
+        <v>279</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="3" t="s">
@@ -5335,33 +5665,33 @@
       </c>
       <c r="N54" s="3"/>
     </row>
-    <row r="55" spans="1:14" ht="15">
+    <row r="55" spans="1:14" ht="27">
       <c r="A55" s="3" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>288</v>
+        <v>262</v>
       </c>
       <c r="C55" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D55" s="4">
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="E55" s="4">
-        <v>46355</v>
+        <v>46348</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="J55" s="3" t="s">
         <v>51</v>
@@ -5377,34 +5707,34 @@
     </row>
     <row r="56" spans="1:14" ht="15">
       <c r="A56" s="3" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>288</v>
+        <v>262</v>
       </c>
       <c r="C56" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D56" s="4">
-        <v>46349</v>
+        <v>46342</v>
       </c>
       <c r="E56" s="4">
-        <v>46355</v>
+        <v>46348</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="3" t="s">
@@ -5417,7 +5747,7 @@
     </row>
     <row r="57" spans="1:14" ht="15">
       <c r="A57" s="3" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>288</v>
@@ -5432,19 +5762,19 @@
         <v>46355</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>294</v>
+        <v>127</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="3" t="s">
@@ -5455,9 +5785,9 @@
       </c>
       <c r="N57" s="3"/>
     </row>
-    <row r="58" spans="1:14" ht="27">
+    <row r="58" spans="1:14" ht="15">
       <c r="A58" s="3" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>288</v>
@@ -5472,16 +5802,16 @@
         <v>46355</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>303</v>
+        <v>287</v>
       </c>
       <c r="J58" s="3" t="s">
         <v>51</v>
@@ -5495,33 +5825,33 @@
       </c>
       <c r="N58" s="3"/>
     </row>
-    <row r="59" spans="1:14" ht="27">
+    <row r="59" spans="1:14" ht="15">
       <c r="A59" s="3" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="C59" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D59" s="4">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="E59" s="4">
-        <v>46362</v>
+        <v>46355</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>140</v>
+        <v>117</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="J59" s="3" t="s">
         <v>113</v>
@@ -5537,31 +5867,31 @@
     </row>
     <row r="60" spans="1:14" ht="15">
       <c r="A60" s="3" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="C60" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D60" s="4">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="E60" s="4">
-        <v>46362</v>
+        <v>46355</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="J60" s="3" t="s">
         <v>113</v>
@@ -5575,36 +5905,36 @@
       </c>
       <c r="N60" s="3"/>
     </row>
-    <row r="61" spans="1:14" ht="15">
+    <row r="61" spans="1:14" ht="27">
       <c r="A61" s="3" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="C61" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D61" s="4">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="E61" s="4">
-        <v>46362</v>
+        <v>46355</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="H61" s="3" t="s">
         <v>117</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="3" t="s">
@@ -5615,485 +5945,1133 @@
       </c>
       <c r="N61" s="3"/>
     </row>
-    <row r="62" spans="1:14" ht="15">
-      <c r="A62" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>305</v>
+    <row r="62" spans="1:14" ht="27">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>B92</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Privacidad</t>
+        </is>
       </c>
       <c r="C62" s="3">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D62" s="4">
-        <v>46356</v>
+        <v>46370</v>
       </c>
       <c r="E62" s="4">
-        <v>46362</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="J62" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K62" s="3"/>
-      <c r="L62" s="3" t="s">
-        <v>54</v>
+        <v>46376</v>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Definir y validar frontera de datos Academy↔Graduate</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Academy solo accede a matrícula, cursos, graduación, certificados y señal autorizada de perfil profesional activo; pruebas de diseño excluyen ventas, clientes, agenda, inventario, ingresos, caja, facturación y datos privados</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>B64-B80</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M62" s="6">
         <v>0</v>
       </c>
-      <c r="N62" s="3"/>
+      <c r="N62" s="3" t="inlineStr">
+        <is>
+          <t>Decisión aprobada; sin comercialización ni intercambio de datos privados</t>
+        </is>
+      </c>
     </row>
     <row r="63" spans="1:14" ht="27">
-      <c r="A63" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>319</v>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>B82</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Core</t>
+        </is>
       </c>
       <c r="C63" s="3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D63" s="4">
-        <v>46363</v>
+        <v>46370</v>
       </c>
       <c r="E63" s="4">
-        <v>46369</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="J63" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K63" s="3"/>
-      <c r="L63" s="3" t="s">
-        <v>54</v>
+        <v>46376</v>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar Academy Core ampliado</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Programas, cursos, módulos, instructores, alumnos, matrículas, progreso y graduación definidos con aislamiento multiempresa/multisucursal</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>B60-B80-B92</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M63" s="6">
         <v>0</v>
       </c>
-      <c r="N63" s="3"/>
+      <c r="N63" s="3" t="inlineStr">
+        <is>
+          <t>Fase posterior al Academy MVP</t>
+        </is>
+      </c>
     </row>
     <row r="64" spans="1:14" ht="27">
-      <c r="A64" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>319</v>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>B83</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Importación</t>
+        </is>
       </c>
       <c r="C64" s="3">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D64" s="4">
-        <v>46363</v>
+        <v>46377</v>
       </c>
       <c r="E64" s="4">
-        <v>46369</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="G64" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I64" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="J64" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K64" s="3"/>
-      <c r="L64" s="3" t="s">
-        <v>54</v>
+        <v>46383</v>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar importación de contenido y alumnos existentes</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Ingreso controlado de PDF, Word, Excel, imágenes y alumnos existentes con trazabilidad, validación y límites</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>B82</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M64" s="6">
         <v>0</v>
       </c>
-      <c r="N64" s="3"/>
-    </row>
-    <row r="65" spans="1:14" ht="15">
-      <c r="A65" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>319</v>
+      <c r="N64" s="3" t="inlineStr">
+        <is>
+          <t>No publicar automáticamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" spans="1:14" ht="27">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>B84</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Importación</t>
+        </is>
       </c>
       <c r="C65" s="3">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D65" s="4">
-        <v>46363</v>
+        <v>46377</v>
       </c>
       <c r="E65" s="4">
-        <v>46369</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="J65" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K65" s="3"/>
-      <c r="L65" s="3" t="s">
-        <v>54</v>
+        <v>46383</v>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar flujo asistido de revisión y aprobación</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Flujo importar→analizar→proponer→revisar→aprobar; ninguna propuesta altera contenido autorizado sin aprobación humana y auditoría</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>B83</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M65" s="6">
         <v>0</v>
       </c>
-      <c r="N65" s="3"/>
-    </row>
-    <row r="66" spans="1:14" ht="15">
-      <c r="A66" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>319</v>
+      <c r="N65" s="3" t="inlineStr">
+        <is>
+          <t>Base para Knowledge AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:14" ht="27">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>B85</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Student Hub</t>
+        </is>
       </c>
       <c r="C66" s="3">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D66" s="4">
-        <v>46363</v>
+        <v>46384</v>
       </c>
       <c r="E66" s="4">
-        <v>46369</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K66" s="3"/>
-      <c r="L66" s="3" t="s">
-        <v>54</v>
+        <v>46390</v>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Planificar Student Hub</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Portal mobile-first de materiales, biblioteca, progreso y certificados validado en móvil/tablet/desktop</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>B82-B84</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M66" s="6">
         <v>0</v>
       </c>
-      <c r="N66" s="3"/>
+      <c r="N66" s="3" t="inlineStr">
+        <is>
+          <t>Flujos móviles pueden ser simplificados</t>
+        </is>
+      </c>
     </row>
     <row r="67" spans="1:14" ht="27">
-      <c r="A67" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>319</v>
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>B86</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Lab</t>
+        </is>
       </c>
       <c r="C67" s="3">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D67" s="4">
-        <v>46363</v>
+        <v>46391</v>
       </c>
       <c r="E67" s="4">
-        <v>46369</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K67" s="3"/>
-      <c r="L67" s="3" t="s">
-        <v>54</v>
+        <v>46397</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar Academy Lab aislado</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Entorno simulado para aprender BeautyOS sin afectar datos reales, con separación explícita de tenants, sucursales y operaciones</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>B82-B85</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
       <c r="M67" s="6">
         <v>0</v>
       </c>
-      <c r="N67" s="3"/>
-    </row>
-    <row r="68" spans="1:14" ht="15">
-      <c r="A68" s="1"/>
-      <c r="B68" s="1"/>
-      <c r="C68" s="1"/>
-      <c r="D68" s="1"/>
-      <c r="E68" s="1"/>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1"/>
-      <c r="H68" s="1"/>
-      <c r="I68" s="1"/>
-      <c r="J68" s="1"/>
-      <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
-    </row>
-    <row r="69" spans="1:14" ht="15">
-      <c r="A69" s="1"/>
-      <c r="B69" s="1"/>
-      <c r="C69" s="1"/>
-      <c r="D69" s="1"/>
-      <c r="E69" s="1"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-      <c r="H69" s="1"/>
-      <c r="I69" s="1"/>
-      <c r="J69" s="1"/>
-      <c r="K69" s="1"/>
-      <c r="L69" s="1"/>
-      <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-    </row>
-    <row r="70" spans="1:14" ht="15">
-      <c r="A70" s="1"/>
-      <c r="B70" s="1"/>
-      <c r="C70" s="1"/>
-      <c r="D70" s="1"/>
-      <c r="E70" s="1"/>
-      <c r="F70" s="1"/>
-      <c r="G70" s="1"/>
-      <c r="H70" s="1"/>
-      <c r="I70" s="1"/>
-      <c r="J70" s="1"/>
-      <c r="K70" s="1"/>
-      <c r="L70" s="1"/>
-      <c r="M70" s="1"/>
-      <c r="N70" s="1"/>
-    </row>
-    <row r="71" spans="1:14" ht="15">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
-      <c r="C71" s="1"/>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-      <c r="I71" s="1"/>
-      <c r="J71" s="1"/>
-      <c r="K71" s="1"/>
-      <c r="L71" s="1"/>
-      <c r="M71" s="1"/>
-      <c r="N71" s="1"/>
-    </row>
-    <row r="72" spans="1:14" ht="15">
-      <c r="A72" s="1"/>
-      <c r="B72" s="1"/>
-      <c r="C72" s="1"/>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="1"/>
-      <c r="I72" s="1"/>
-      <c r="J72" s="1"/>
-      <c r="K72" s="1"/>
-      <c r="L72" s="1"/>
-      <c r="M72" s="1"/>
-      <c r="N72" s="1"/>
-    </row>
-    <row r="73" spans="1:14" ht="15">
-      <c r="A73" s="1"/>
-      <c r="B73" s="1"/>
-      <c r="C73" s="1"/>
-      <c r="D73" s="1"/>
-      <c r="E73" s="1"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1"/>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1"/>
-      <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
+      <c r="N67" s="3" t="inlineStr">
+        <is>
+          <t>Datos simulados claramente identificados</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:14" ht="27">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>B87</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Certificación</t>
+        </is>
+      </c>
+      <c r="C68" s="3">
+        <v>21</v>
+      </c>
+      <c r="D68" s="4">
+        <v>46398</v>
+      </c>
+      <c r="E68" s="4">
+        <v>46404</v>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar certificaciones verificables</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Certificados verificables, revocables, con emisor, versión, evidencia y exposición pública mínima sin filtrar datos educativos privados</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>B82-B85</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M68" s="6">
+        <v>0</v>
+      </c>
+      <c r="N68" s="3" t="inlineStr">
+        <is>
+          <t>Respeta consentimiento y privacidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="27">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>B88</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Graduados</t>
+        </is>
+      </c>
+      <c r="C69" s="3">
+        <v>22</v>
+      </c>
+      <c r="D69" s="4">
+        <v>46405</v>
+      </c>
+      <c r="E69" s="4">
+        <v>46411</v>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar Graduate Network y continuidad de identidad</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Red de graduados opt-in y transición Student→Graduate→Professional sin duplicar User ni transferir datos privados del negocio a Academy</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>B63-B87-B92</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M69" s="6">
+        <v>0</v>
+      </c>
+      <c r="N69" s="3" t="inlineStr">
+        <is>
+          <t>Activación profesional voluntaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="27">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>B89</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Knowledge AI</t>
+        </is>
+      </c>
+      <c r="C70" s="3">
+        <v>23</v>
+      </c>
+      <c r="D70" s="4">
+        <v>46412</v>
+      </c>
+      <c r="E70" s="4">
+        <v>46418</v>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar Knowledge AI sobre contenido autorizado</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Respuestas con fuente y versión; solo contenido autorizado; permisos, trazabilidad, revisión y retiro de fuentes definidos</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>B84-B85</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M70" s="6">
+        <v>0</v>
+      </c>
+      <c r="N70" s="3" t="inlineStr">
+        <is>
+          <t>IA no es fuente de verdad</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:14" ht="27">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>B90</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Brand Knowledge</t>
+        </is>
+      </c>
+      <c r="C71" s="3">
+        <v>23</v>
+      </c>
+      <c r="D71" s="4">
+        <v>46412</v>
+      </c>
+      <c r="E71" s="4">
+        <v>46418</v>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar Brand Knowledge verificable</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Marcas, líneas, productos, fichas, procedimientos y contenido oficial/verificado con procedencia, vigencia y versionado</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>B84</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M71" s="6">
+        <v>0</v>
+      </c>
+      <c r="N71" s="3" t="inlineStr">
+        <is>
+          <t>Distinguir contenido oficial, verificado y no verificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:14" ht="27">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>B91</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Academy — Templates</t>
+        </is>
+      </c>
+      <c r="C72" s="3">
+        <v>24</v>
+      </c>
+      <c r="D72" s="4">
+        <v>46419</v>
+      </c>
+      <c r="E72" s="4">
+        <v>46425</v>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Diseñar BeautyOS Templates propios</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Biblioteca propia de plantillas con procedencia y licencia; prohibido reutilizar contenido privado de academias para crear plantillas generales</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>B89-B90</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M72" s="6">
+        <v>0</v>
+      </c>
+      <c r="N72" s="3" t="inlineStr">
+        <is>
+          <t>Separación estricta de propiedad intelectual y privacidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="27">
+      <c r="A73" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C73" s="3">
+        <v>15</v>
+      </c>
+      <c r="D73" s="4">
+        <v>46356</v>
+      </c>
+      <c r="E73" s="4">
+        <v>46362</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M73" s="6">
+        <v>0</v>
+      </c>
+      <c r="N73" s="3"/>
     </row>
     <row r="74" spans="1:14" ht="15">
-      <c r="A74" s="1"/>
-      <c r="B74" s="1"/>
-      <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1"/>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1"/>
-      <c r="M74" s="1"/>
-      <c r="N74" s="1"/>
+      <c r="A74" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C74" s="3">
+        <v>15</v>
+      </c>
+      <c r="D74" s="4">
+        <v>46356</v>
+      </c>
+      <c r="E74" s="4">
+        <v>46362</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M74" s="6">
+        <v>0</v>
+      </c>
+      <c r="N74" s="3"/>
     </row>
     <row r="75" spans="1:14" ht="15">
-      <c r="A75" s="1"/>
-      <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-      <c r="I75" s="1"/>
-      <c r="J75" s="1"/>
-      <c r="K75" s="1"/>
-      <c r="L75" s="1"/>
-      <c r="M75" s="1"/>
-      <c r="N75" s="1"/>
+      <c r="A75" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C75" s="3">
+        <v>15</v>
+      </c>
+      <c r="D75" s="4">
+        <v>46356</v>
+      </c>
+      <c r="E75" s="4">
+        <v>46362</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M75" s="6">
+        <v>0</v>
+      </c>
+      <c r="N75" s="3"/>
     </row>
     <row r="76" spans="1:14" ht="15">
-      <c r="A76" s="1"/>
-      <c r="B76" s="1"/>
-      <c r="C76" s="1"/>
-      <c r="D76" s="1"/>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1"/>
-      <c r="K76" s="1"/>
-      <c r="L76" s="1"/>
-      <c r="M76" s="1"/>
-      <c r="N76" s="1"/>
-    </row>
-    <row r="77" spans="1:14" ht="15">
-      <c r="A77" s="1"/>
-      <c r="B77" s="1"/>
-      <c r="C77" s="1"/>
-      <c r="D77" s="1"/>
-      <c r="E77" s="1"/>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="1"/>
-      <c r="I77" s="1"/>
-      <c r="J77" s="1"/>
-      <c r="K77" s="1"/>
-      <c r="L77" s="1"/>
-      <c r="M77" s="1"/>
-      <c r="N77" s="1"/>
-    </row>
-    <row r="78" spans="1:14" ht="15">
-      <c r="A78" s="1"/>
-      <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
-      <c r="D78" s="1"/>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-      <c r="H78" s="1"/>
-      <c r="I78" s="1"/>
-      <c r="J78" s="1"/>
-      <c r="K78" s="1"/>
-      <c r="L78" s="1"/>
-      <c r="M78" s="1"/>
-      <c r="N78" s="1"/>
+      <c r="A76" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C76" s="3">
+        <v>15</v>
+      </c>
+      <c r="D76" s="4">
+        <v>46356</v>
+      </c>
+      <c r="E76" s="4">
+        <v>46362</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M76" s="6">
+        <v>0</v>
+      </c>
+      <c r="N76" s="3"/>
+    </row>
+    <row r="77" spans="1:14" ht="27">
+      <c r="A77" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C77" s="3">
+        <v>16</v>
+      </c>
+      <c r="D77" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E77" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M77" s="6">
+        <v>0</v>
+      </c>
+      <c r="N77" s="3"/>
+    </row>
+    <row r="78" spans="1:14" ht="27">
+      <c r="A78" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C78" s="3">
+        <v>16</v>
+      </c>
+      <c r="D78" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E78" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M78" s="6">
+        <v>0</v>
+      </c>
+      <c r="N78" s="3"/>
     </row>
     <row r="79" spans="1:14" ht="15">
-      <c r="A79" s="1"/>
-      <c r="B79" s="1"/>
-      <c r="C79" s="1"/>
-      <c r="D79" s="1"/>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-      <c r="H79" s="1"/>
-      <c r="I79" s="1"/>
-      <c r="J79" s="1"/>
-      <c r="K79" s="1"/>
-      <c r="L79" s="1"/>
-      <c r="M79" s="1"/>
-      <c r="N79" s="1"/>
-    </row>
-    <row r="80" spans="1:14" ht="15">
-      <c r="A80" s="1"/>
-      <c r="B80" s="1"/>
-      <c r="C80" s="1"/>
-      <c r="D80" s="1"/>
-      <c r="E80" s="1"/>
-      <c r="F80" s="1"/>
-      <c r="G80" s="1"/>
-      <c r="H80" s="1"/>
-      <c r="I80" s="1"/>
-      <c r="J80" s="1"/>
-      <c r="K80" s="1"/>
-      <c r="L80" s="1"/>
-      <c r="M80" s="1"/>
-      <c r="N80" s="1"/>
+      <c r="A79" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C79" s="3">
+        <v>16</v>
+      </c>
+      <c r="D79" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E79" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M79" s="6">
+        <v>0</v>
+      </c>
+      <c r="N79" s="3"/>
+    </row>
+    <row r="80" spans="1:14" ht="27">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>B93</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Comercial — Academy</t>
+        </is>
+      </c>
+      <c r="C80" s="3">
+        <v>16</v>
+      </c>
+      <c r="D80" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E80" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Validar hipótesis Academy Founder/Partner</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Experimento aprobado o descartado para primer año gratis/subsidiado, límites de almacenamiento/IA y créditos por activación profesional voluntaria, con costos, anti-abuso y privacidad medidos</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>B64-B74-B76-B92</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M80" s="6">
+        <v>0</v>
+      </c>
+      <c r="N80" s="3" t="inlineStr">
+        <is>
+          <t>HIPÓTESIS; no constituye precio, beneficio ni acuerdo definitivo</t>
+        </is>
+      </c>
     </row>
     <row r="81" spans="1:14" ht="15">
-      <c r="A81" s="1"/>
-      <c r="B81" s="1"/>
-      <c r="C81" s="1"/>
-      <c r="D81" s="1"/>
-      <c r="E81" s="1"/>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="H81" s="1"/>
-      <c r="I81" s="1"/>
-      <c r="J81" s="1"/>
-      <c r="K81" s="1"/>
-      <c r="L81" s="1"/>
-      <c r="M81" s="1"/>
-      <c r="N81" s="1"/>
-    </row>
-    <row r="82" spans="1:14" ht="15">
-      <c r="A82" s="1"/>
-      <c r="B82" s="1"/>
-      <c r="C82" s="1"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1"/>
-      <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="1"/>
-      <c r="L82" s="1"/>
-      <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
+      <c r="A81" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C81" s="3">
+        <v>16</v>
+      </c>
+      <c r="D81" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E81" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K81" s="3"/>
+      <c r="L81" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M81" s="6">
+        <v>0</v>
+      </c>
+      <c r="N81" s="3"/>
+    </row>
+    <row r="82" spans="1:14" ht="27">
+      <c r="A82" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C82" s="3">
+        <v>16</v>
+      </c>
+      <c r="D82" s="4">
+        <v>46363</v>
+      </c>
+      <c r="E82" s="4">
+        <v>46369</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K82" s="3"/>
+      <c r="L82" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="M82" s="6">
+        <v>0</v>
+      </c>
+      <c r="N82" s="3"/>
     </row>
     <row r="83" spans="1:14" ht="15">
       <c r="A83" s="1"/>
@@ -6382,6 +7360,246 @@
       <c r="L100" s="1"/>
       <c r="M100" s="1"/>
       <c r="N100" s="1"/>
+    </row>
+    <row r="101" spans="1:14" ht="15">
+      <c r="A101" s="1"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="1"/>
+      <c r="I101" s="1"/>
+      <c r="J101" s="1"/>
+      <c r="K101" s="1"/>
+      <c r="L101" s="1"/>
+      <c r="M101" s="1"/>
+      <c r="N101" s="1"/>
+    </row>
+    <row r="102" spans="1:14" ht="15">
+      <c r="A102" s="1"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="1"/>
+      <c r="I102" s="1"/>
+      <c r="J102" s="1"/>
+      <c r="K102" s="1"/>
+      <c r="L102" s="1"/>
+      <c r="M102" s="1"/>
+      <c r="N102" s="1"/>
+    </row>
+    <row r="103" spans="1:14" ht="15">
+      <c r="A103" s="1"/>
+      <c r="B103" s="1"/>
+      <c r="C103" s="1"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="1"/>
+      <c r="I103" s="1"/>
+      <c r="J103" s="1"/>
+      <c r="K103" s="1"/>
+      <c r="L103" s="1"/>
+      <c r="M103" s="1"/>
+      <c r="N103" s="1"/>
+    </row>
+    <row r="104" spans="1:14" ht="15">
+      <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
+      <c r="J104" s="1"/>
+      <c r="K104" s="1"/>
+      <c r="L104" s="1"/>
+      <c r="M104" s="1"/>
+      <c r="N104" s="1"/>
+    </row>
+    <row r="105" spans="1:14" ht="15">
+      <c r="A105" s="1"/>
+      <c r="B105" s="1"/>
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1"/>
+      <c r="F105" s="1"/>
+      <c r="G105" s="1"/>
+      <c r="H105" s="1"/>
+      <c r="I105" s="1"/>
+      <c r="J105" s="1"/>
+      <c r="K105" s="1"/>
+      <c r="L105" s="1"/>
+      <c r="M105" s="1"/>
+      <c r="N105" s="1"/>
+    </row>
+    <row r="106" spans="1:14" ht="15">
+      <c r="A106" s="1"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="1"/>
+      <c r="G106" s="1"/>
+      <c r="H106" s="1"/>
+      <c r="I106" s="1"/>
+      <c r="J106" s="1"/>
+      <c r="K106" s="1"/>
+      <c r="L106" s="1"/>
+      <c r="M106" s="1"/>
+      <c r="N106" s="1"/>
+    </row>
+    <row r="107" spans="1:14" ht="15">
+      <c r="A107" s="1"/>
+      <c r="B107" s="1"/>
+      <c r="C107" s="1"/>
+      <c r="D107" s="1"/>
+      <c r="E107" s="1"/>
+      <c r="F107" s="1"/>
+      <c r="G107" s="1"/>
+      <c r="H107" s="1"/>
+      <c r="I107" s="1"/>
+      <c r="J107" s="1"/>
+      <c r="K107" s="1"/>
+      <c r="L107" s="1"/>
+      <c r="M107" s="1"/>
+      <c r="N107" s="1"/>
+    </row>
+    <row r="108" spans="1:14" ht="15">
+      <c r="A108" s="1"/>
+      <c r="B108" s="1"/>
+      <c r="C108" s="1"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+      <c r="F108" s="1"/>
+      <c r="G108" s="1"/>
+      <c r="H108" s="1"/>
+      <c r="I108" s="1"/>
+      <c r="J108" s="1"/>
+      <c r="K108" s="1"/>
+      <c r="L108" s="1"/>
+      <c r="M108" s="1"/>
+      <c r="N108" s="1"/>
+    </row>
+    <row r="109" spans="1:14" ht="15">
+      <c r="A109" s="1"/>
+      <c r="B109" s="1"/>
+      <c r="C109" s="1"/>
+      <c r="D109" s="1"/>
+      <c r="E109" s="1"/>
+      <c r="F109" s="1"/>
+      <c r="G109" s="1"/>
+      <c r="H109" s="1"/>
+      <c r="I109" s="1"/>
+      <c r="J109" s="1"/>
+      <c r="K109" s="1"/>
+      <c r="L109" s="1"/>
+      <c r="M109" s="1"/>
+      <c r="N109" s="1"/>
+    </row>
+    <row r="110" spans="1:14" ht="15">
+      <c r="A110" s="1"/>
+      <c r="B110" s="1"/>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="1"/>
+      <c r="H110" s="1"/>
+      <c r="I110" s="1"/>
+      <c r="J110" s="1"/>
+      <c r="K110" s="1"/>
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+      <c r="N110" s="1"/>
+    </row>
+    <row r="111" spans="1:14" ht="15">
+      <c r="A111" s="1"/>
+      <c r="B111" s="1"/>
+      <c r="C111" s="1"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="1"/>
+      <c r="H111" s="1"/>
+      <c r="I111" s="1"/>
+      <c r="J111" s="1"/>
+      <c r="K111" s="1"/>
+      <c r="L111" s="1"/>
+      <c r="M111" s="1"/>
+      <c r="N111" s="1"/>
+    </row>
+    <row r="112" spans="1:14" ht="15">
+      <c r="A112" s="1"/>
+      <c r="B112" s="1"/>
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="1"/>
+      <c r="G112" s="1"/>
+      <c r="H112" s="1"/>
+      <c r="I112" s="1"/>
+      <c r="J112" s="1"/>
+      <c r="K112" s="1"/>
+      <c r="L112" s="1"/>
+      <c r="M112" s="1"/>
+      <c r="N112" s="1"/>
+    </row>
+    <row r="113" spans="1:14" ht="15">
+      <c r="A113" s="1"/>
+      <c r="B113" s="1"/>
+      <c r="C113" s="1"/>
+      <c r="D113" s="1"/>
+      <c r="E113" s="1"/>
+      <c r="F113" s="1"/>
+      <c r="G113" s="1"/>
+      <c r="H113" s="1"/>
+      <c r="I113" s="1"/>
+      <c r="J113" s="1"/>
+      <c r="K113" s="1"/>
+      <c r="L113" s="1"/>
+      <c r="M113" s="1"/>
+      <c r="N113" s="1"/>
+    </row>
+    <row r="114" spans="1:14" ht="15">
+      <c r="A114" s="1"/>
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+      <c r="F114" s="1"/>
+      <c r="G114" s="1"/>
+      <c r="H114" s="1"/>
+      <c r="I114" s="1"/>
+      <c r="J114" s="1"/>
+      <c r="K114" s="1"/>
+      <c r="L114" s="1"/>
+      <c r="M114" s="1"/>
+      <c r="N114" s="1"/>
+    </row>
+    <row r="115" spans="1:14" ht="15">
+      <c r="A115" s="1"/>
+      <c r="B115" s="1"/>
+      <c r="C115" s="1"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="1"/>
+      <c r="F115" s="1"/>
+      <c r="G115" s="1"/>
+      <c r="H115" s="1"/>
+      <c r="I115" s="1"/>
+      <c r="J115" s="1"/>
+      <c r="K115" s="1"/>
+      <c r="L115" s="1"/>
+      <c r="M115" s="1"/>
+      <c r="N115" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8717,8 +9935,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
-        <v>533</v>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Modelo comercial — HIPÓTESIS para validación, no precios definitivos</t>
+        </is>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8876,17 +10096,25 @@
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:9" ht="27">
-      <c r="A8" s="3" t="s">
-        <v>566</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>568</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>569</v>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Academy Founder/Partner</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>BeautyOS Academy (hipótesis)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Academy Core + Student Hub + Lab + certificación, sujeto a fases y límites</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Posible primer año gratis/subsidiado; por validar</t>
+        </is>
       </c>
       <c r="E8" s="3" t="s">
         <v>92</v>
@@ -8894,11 +10122,15 @@
       <c r="F8" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>570</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>571</v>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Canal educativo y activación profesional voluntaria</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Definir costos, almacenamiento, IA, elegibilidad y anti-abuso</t>
+        </is>
       </c>
       <c r="I8" s="1"/>
     </row>
@@ -9026,37 +10258,145 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" ht="15">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Límites almacenamiento/IA</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>HIPÓTESIS: cuotas o uso medido que protejan sostenibilidad y privacidad.</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Créditos por activación</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>HIPÓTESIS: créditos si graduados activan voluntariamente BeautyOS Professional; sin vender ni intercambiar datos privados.</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="15">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Privacidad no negociable</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Nunca comercializar ni intercambiar datos privados de alumnos, graduados, profesionales o sus negocios.</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="15">
       <c r="A21" s="1"/>
@@ -9475,9 +10815,15 @@
       <c r="E4" s="3" t="s">
         <v>594</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
-        <v>54</v>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Compartir/reutilizar Core; BeautyOS independiente de módulos exclusivos MVS</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -9613,9 +10959,15 @@
       <c r="E10" s="3" t="s">
         <v>617</v>
       </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3" t="s">
-        <v>54</v>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Mantener como hipótesis; validar sostenibilidad, límites y privacidad</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hipótesis</t>
+        </is>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -9659,9 +11011,15 @@
       <c r="E12" s="3" t="s">
         <v>598</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3" t="s">
-        <v>54</v>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Web/PWA mobile-first; validar móvil/tablet/desktop y permitir flujos móviles simplificados</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -9690,59 +11048,239 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:9" ht="15">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>¿Qué identidad usan Student, Professional e Instructor?</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Un User Core; perfiles/relaciones sin identidades duplicadas</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Muy alto</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Antes de Academy Core</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="15">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>¿Qué datos puede conocer Academy del negocio de un egresado?</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Solo relación educativa y señal autorizada de perfil activo</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Muy alto</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Antes de Academy Core</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Aprobado; exclusión explícita de datos privados del negocio</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="15">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>¿Academy Founder/Partner y créditos son condiciones definitivas?</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>No; son hipótesis sujetas a validación</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Antes de oferta comercial</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Validar costos, límites, elegibilidad y anti-abuso</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Hipótesis</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="15">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>¿Knowledge AI puede usar contenido no autorizado o privado?</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>No; solo contenido autorizado con fuente y versión</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Muy alto</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Antes de Knowledge AI</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="15">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>¿BeautyOS Templates puede derivarse de contenido privado de academias?</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>No; plantillas propias con procedencia/licencia</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Muy alto</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Antes de Templates</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15">
       <c r="A19" s="1"/>

</xml_diff>

<commit_message>
wip: preservar avance parcial B10
</commit_message>
<xml_diff>
--- a/docs/beautyos/BeautyOS_Cronograma_Maestro.xlsx
+++ b/docs/beautyos/BeautyOS_Cronograma_Maestro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\MVS Commerce\Proyecto POS MVS\mvs-commerce-beautyos\docs\beautyos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB9AC0B-5933-4FD1-8915-2F53555F970B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CEF3C5-A054-47E2-AA07-C36EC12E4D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2940" yWindow="2940" windowWidth="15375" windowHeight="7785" tabRatio="737" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1417" uniqueCount="779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="780">
   <si>
     <t>BeautyOS — Cronograma Maestro de Trabajo</t>
   </si>
@@ -2350,9 +2350,6 @@
     <t>Siguiente tarea</t>
   </si>
   <si>
-    <t>B10 — Crear módulo de profesionales. No iniciado por la aprobación de B09.</t>
-  </si>
-  <si>
     <t>Portal inicial sin contraseña obligatoria; acceso seguro por token/QR.</t>
   </si>
   <si>
@@ -2363,6 +2360,12 @@
   </si>
   <si>
     <t>Estética usa servicios/citas base en MVP; sesiones/paquetes especializados quedan Post-MVP.</t>
+  </si>
+  <si>
+    <t>CRUD mobile-first de perfiles Professional sobre User Core; scopes por empresa/sucursal, permisos, asignación de sucursales/especialidades y aislamiento cross-company. Evidencia: BeautyProfessionalManagementTest (8 pruebas, 34 aserciones).</t>
+  </si>
+  <si>
+    <t>B11 — Crear catálogo de servicios. No iniciado.</t>
   </si>
 </sst>
 </file>
@@ -2477,6 +2480,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2484,21 +2494,11 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2587,6 +2587,9 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2617,7 +2620,7 @@
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Estado"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="% avance"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Observaciones"/>
-    <tableColumn id="15" xr3:uid="{7B52D3BE-2311-4EC9-853D-6D16269D1BFE}" name="Clasificación B09" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{7B52D3BE-2311-4EC9-853D-6D16269D1BFE}" name="Clasificación B09" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2877,16 +2880,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="15">
@@ -2908,13 +2911,13 @@
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="40.5">
@@ -3581,7 +3584,7 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" ht="15">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="10" t="s">
         <v>770</v>
       </c>
       <c r="B33" s="1"/>
@@ -3628,7 +3631,7 @@
         <v>773</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -3798,10 +3801,10 @@
     <mergeCell ref="D3:H3"/>
   </mergeCells>
   <conditionalFormatting sqref="H14:H20">
-    <cfRule type="expression" dxfId="8" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>H14="Completado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>H14="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3831,26 +3834,26 @@
     <col min="11" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
     <col min="14" max="14" width="30" customWidth="1"/>
-    <col min="15" max="15" width="16.625" style="11" customWidth="1"/>
+    <col min="15" max="15" width="16.625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
     </row>
     <row r="2" spans="1:15" ht="15">
       <c r="A2" s="1"/>
@@ -3911,7 +3914,7 @@
       <c r="N3" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="9" t="s">
         <v>753</v>
       </c>
     </row>
@@ -3954,7 +3957,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="3"/>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -3997,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="3"/>
-      <c r="O5" s="11" t="s">
+      <c r="O5" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4040,7 +4043,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="3"/>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4083,7 +4086,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="3"/>
-      <c r="O7" s="11" t="s">
+      <c r="O7" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4126,7 +4129,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="3"/>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4171,7 +4174,7 @@
       <c r="N9" s="3" t="s">
         <v>754</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="O9" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4216,7 +4219,7 @@
       <c r="N10" s="3" t="s">
         <v>758</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4261,7 +4264,7 @@
       <c r="N11" s="3" t="s">
         <v>756</v>
       </c>
-      <c r="O11" s="11" t="s">
+      <c r="O11" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4306,7 +4309,7 @@
       <c r="N12" s="3" t="s">
         <v>757</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="O12" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4351,7 +4354,7 @@
       <c r="N13" s="3" t="s">
         <v>755</v>
       </c>
-      <c r="O13" s="11" t="s">
+      <c r="O13" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4398,7 +4401,7 @@
       <c r="N14" s="3" t="s">
         <v>623</v>
       </c>
-      <c r="O14" s="11" t="s">
+      <c r="O14" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4445,7 +4448,7 @@
       <c r="N15" s="3" t="s">
         <v>628</v>
       </c>
-      <c r="O15" s="11" t="s">
+      <c r="O15" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4492,11 +4495,11 @@
       <c r="N16" s="3" t="s">
         <v>633</v>
       </c>
-      <c r="O16" s="11" t="s">
+      <c r="O16" s="8" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="15">
+    <row r="17" spans="1:15" ht="94.5">
       <c r="A17" s="3" t="s">
         <v>145</v>
       </c>
@@ -4529,13 +4532,15 @@
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="s">
-        <v>54</v>
+        <v>616</v>
       </c>
       <c r="M17" s="6">
-        <v>0</v>
-      </c>
-      <c r="N17" s="3"/>
-      <c r="O17" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="O17" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4578,7 +4583,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="3"/>
-      <c r="O18" s="11" t="s">
+      <c r="O18" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4621,7 +4626,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="3"/>
-      <c r="O19" s="11" t="s">
+      <c r="O19" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4664,7 +4669,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="3"/>
-      <c r="O20" s="11" t="s">
+      <c r="O20" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4707,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="N21" s="3"/>
-      <c r="O21" s="11" t="s">
+      <c r="O21" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4750,7 +4755,7 @@
         <v>0</v>
       </c>
       <c r="N22" s="3"/>
-      <c r="O22" s="11" t="s">
+      <c r="O22" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4793,7 +4798,7 @@
         <v>0</v>
       </c>
       <c r="N23" s="3"/>
-      <c r="O23" s="11" t="s">
+      <c r="O23" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4836,7 +4841,7 @@
         <v>0</v>
       </c>
       <c r="N24" s="3"/>
-      <c r="O24" s="11" t="s">
+      <c r="O24" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4879,7 +4884,7 @@
         <v>0</v>
       </c>
       <c r="N25" s="3"/>
-      <c r="O25" s="11" t="s">
+      <c r="O25" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4922,7 +4927,7 @@
         <v>0</v>
       </c>
       <c r="N26" s="3"/>
-      <c r="O26" s="11" t="s">
+      <c r="O26" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -4965,7 +4970,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="3"/>
-      <c r="O27" s="11" t="s">
+      <c r="O27" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5008,7 +5013,7 @@
         <v>0</v>
       </c>
       <c r="N28" s="3"/>
-      <c r="O28" s="11" t="s">
+      <c r="O28" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5051,7 +5056,7 @@
         <v>0</v>
       </c>
       <c r="N29" s="3"/>
-      <c r="O29" s="11" t="s">
+      <c r="O29" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5094,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="N30" s="3"/>
-      <c r="O30" s="11" t="s">
+      <c r="O30" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5137,7 +5142,7 @@
         <v>0</v>
       </c>
       <c r="N31" s="3"/>
-      <c r="O31" s="11" t="s">
+      <c r="O31" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5180,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="3"/>
-      <c r="O32" s="11" t="s">
+      <c r="O32" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5223,7 +5228,7 @@
         <v>0</v>
       </c>
       <c r="N33" s="3"/>
-      <c r="O33" s="11" t="s">
+      <c r="O33" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5266,7 +5271,7 @@
         <v>0</v>
       </c>
       <c r="N34" s="3"/>
-      <c r="O34" s="11" t="s">
+      <c r="O34" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5309,7 +5314,7 @@
         <v>0</v>
       </c>
       <c r="N35" s="3"/>
-      <c r="O35" s="11" t="s">
+      <c r="O35" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5352,7 +5357,7 @@
         <v>0</v>
       </c>
       <c r="N36" s="3"/>
-      <c r="O36" s="11" t="s">
+      <c r="O36" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5395,7 +5400,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="3"/>
-      <c r="O37" s="11" t="s">
+      <c r="O37" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5438,7 +5443,7 @@
         <v>0</v>
       </c>
       <c r="N38" s="3"/>
-      <c r="O38" s="11" t="s">
+      <c r="O38" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5481,7 +5486,7 @@
         <v>0</v>
       </c>
       <c r="N39" s="3"/>
-      <c r="O39" s="11" t="s">
+      <c r="O39" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5524,7 +5529,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="3"/>
-      <c r="O40" s="11" t="s">
+      <c r="O40" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5567,7 +5572,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="3"/>
-      <c r="O41" s="11" t="s">
+      <c r="O41" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5610,7 +5615,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="3"/>
-      <c r="O42" s="11" t="s">
+      <c r="O42" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5653,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="N43" s="3"/>
-      <c r="O43" s="11" t="s">
+      <c r="O43" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5696,7 +5701,7 @@
         <v>0</v>
       </c>
       <c r="N44" s="3"/>
-      <c r="O44" s="11" t="s">
+      <c r="O44" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5739,7 +5744,7 @@
         <v>0</v>
       </c>
       <c r="N45" s="3"/>
-      <c r="O45" s="11" t="s">
+      <c r="O45" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5782,7 +5787,7 @@
         <v>0</v>
       </c>
       <c r="N46" s="3"/>
-      <c r="O46" s="11" t="s">
+      <c r="O46" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5825,7 +5830,7 @@
         <v>0</v>
       </c>
       <c r="N47" s="3"/>
-      <c r="O47" s="11" t="s">
+      <c r="O47" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5868,7 +5873,7 @@
         <v>0</v>
       </c>
       <c r="N48" s="3"/>
-      <c r="O48" s="11" t="s">
+      <c r="O48" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5911,7 +5916,7 @@
         <v>0</v>
       </c>
       <c r="N49" s="3"/>
-      <c r="O49" s="11" t="s">
+      <c r="O49" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5954,7 +5959,7 @@
         <v>0</v>
       </c>
       <c r="N50" s="3"/>
-      <c r="O50" s="11" t="s">
+      <c r="O50" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -5997,7 +6002,7 @@
         <v>0</v>
       </c>
       <c r="N51" s="3"/>
-      <c r="O51" s="11" t="s">
+      <c r="O51" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6040,7 +6045,7 @@
         <v>0</v>
       </c>
       <c r="N52" s="3"/>
-      <c r="O52" s="11" t="s">
+      <c r="O52" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6083,7 +6088,7 @@
         <v>0</v>
       </c>
       <c r="N53" s="3"/>
-      <c r="O53" s="11" t="s">
+      <c r="O53" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6126,7 +6131,7 @@
         <v>0</v>
       </c>
       <c r="N54" s="3"/>
-      <c r="O54" s="11" t="s">
+      <c r="O54" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6169,7 +6174,7 @@
         <v>0</v>
       </c>
       <c r="N55" s="3"/>
-      <c r="O55" s="11" t="s">
+      <c r="O55" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6212,7 +6217,7 @@
         <v>0</v>
       </c>
       <c r="N56" s="3"/>
-      <c r="O56" s="11" t="s">
+      <c r="O56" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6255,7 +6260,7 @@
         <v>0</v>
       </c>
       <c r="N57" s="3"/>
-      <c r="O57" s="11" t="s">
+      <c r="O57" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6298,7 +6303,7 @@
         <v>0</v>
       </c>
       <c r="N58" s="3"/>
-      <c r="O58" s="11" t="s">
+      <c r="O58" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6341,7 +6346,7 @@
         <v>0</v>
       </c>
       <c r="N59" s="3"/>
-      <c r="O59" s="11" t="s">
+      <c r="O59" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6384,7 +6389,7 @@
         <v>0</v>
       </c>
       <c r="N60" s="3"/>
-      <c r="O60" s="11" t="s">
+      <c r="O60" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6427,7 +6432,7 @@
         <v>0</v>
       </c>
       <c r="N61" s="3"/>
-      <c r="O61" s="11" t="s">
+      <c r="O61" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6474,7 +6479,7 @@
       <c r="N62" s="3" t="s">
         <v>639</v>
       </c>
-      <c r="O62" s="11" t="s">
+      <c r="O62" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6521,7 +6526,7 @@
       <c r="N63" s="3" t="s">
         <v>645</v>
       </c>
-      <c r="O63" s="11" t="s">
+      <c r="O63" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6568,7 +6573,7 @@
       <c r="N64" s="3" t="s">
         <v>650</v>
       </c>
-      <c r="O64" s="11" t="s">
+      <c r="O64" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6615,7 +6620,7 @@
       <c r="N65" s="3" t="s">
         <v>654</v>
       </c>
-      <c r="O65" s="11" t="s">
+      <c r="O65" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6662,7 +6667,7 @@
       <c r="N66" s="3" t="s">
         <v>660</v>
       </c>
-      <c r="O66" s="11" t="s">
+      <c r="O66" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6709,7 +6714,7 @@
       <c r="N67" s="3" t="s">
         <v>666</v>
       </c>
-      <c r="O67" s="11" t="s">
+      <c r="O67" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6756,7 +6761,7 @@
       <c r="N68" s="3" t="s">
         <v>671</v>
       </c>
-      <c r="O68" s="11" t="s">
+      <c r="O68" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6803,7 +6808,7 @@
       <c r="N69" s="3" t="s">
         <v>677</v>
       </c>
-      <c r="O69" s="11" t="s">
+      <c r="O69" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6850,7 +6855,7 @@
       <c r="N70" s="3" t="s">
         <v>683</v>
       </c>
-      <c r="O70" s="11" t="s">
+      <c r="O70" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6897,7 +6902,7 @@
       <c r="N71" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="O71" s="11" t="s">
+      <c r="O71" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6944,7 +6949,7 @@
       <c r="N72" s="3" t="s">
         <v>694</v>
       </c>
-      <c r="O72" s="11" t="s">
+      <c r="O72" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -6989,7 +6994,7 @@
       <c r="N73" s="3" t="s">
         <v>762</v>
       </c>
-      <c r="O73" s="11" t="s">
+      <c r="O73" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7032,7 +7037,7 @@
         <v>0</v>
       </c>
       <c r="N74" s="3"/>
-      <c r="O74" s="11" t="s">
+      <c r="O74" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7075,7 +7080,7 @@
         <v>0</v>
       </c>
       <c r="N75" s="3"/>
-      <c r="O75" s="11" t="s">
+      <c r="O75" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7118,7 +7123,7 @@
         <v>0</v>
       </c>
       <c r="N76" s="3"/>
-      <c r="O76" s="11" t="s">
+      <c r="O76" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7163,7 +7168,7 @@
       <c r="N77" s="3" t="s">
         <v>765</v>
       </c>
-      <c r="O77" s="11" t="s">
+      <c r="O77" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7208,7 +7213,7 @@
       <c r="N78" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="O78" s="11" t="s">
+      <c r="O78" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -7253,7 +7258,7 @@
       <c r="N79" s="3" t="s">
         <v>767</v>
       </c>
-      <c r="O79" s="11" t="s">
+      <c r="O79" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -7300,7 +7305,7 @@
       <c r="N80" s="3" t="s">
         <v>700</v>
       </c>
-      <c r="O80" s="11" t="s">
+      <c r="O80" s="8" t="s">
         <v>614</v>
       </c>
     </row>
@@ -7345,7 +7350,7 @@
       <c r="N81" s="3" t="s">
         <v>768</v>
       </c>
-      <c r="O81" s="11" t="s">
+      <c r="O81" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7390,7 +7395,7 @@
       <c r="N82" s="3" t="s">
         <v>769</v>
       </c>
-      <c r="O82" s="11" t="s">
+      <c r="O82" s="8" t="s">
         <v>416</v>
       </c>
     </row>
@@ -7927,10 +7932,10 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="L4:L67">
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>L4="Completado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>L4="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8003,16 +8008,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="15">
@@ -8799,10 +8804,10 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="H4:H17">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>H4="Completado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>H4="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8834,17 +8839,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>408</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" ht="15">
       <c r="A2" s="1"/>
@@ -9567,16 +9572,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>478</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="15">
@@ -10256,16 +10261,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>713</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" ht="15">
@@ -11004,15 +11009,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>570</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
@@ -11094,7 +11099,7 @@
         <v>584</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>727</v>
@@ -11119,7 +11124,7 @@
         <v>584</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>727</v>
@@ -11144,7 +11149,7 @@
         <v>591</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>727</v>
@@ -11169,7 +11174,7 @@
         <v>595</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>727</v>
@@ -11798,10 +11803,10 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="G4:G13">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>G4="Completado"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>G4="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>